<commit_message>
thêm chức năng search nội dung trong danh sách
</commit_message>
<xml_diff>
--- a/src/OngGio.Infrastructure/Templates/BaoGiaExportTemplate.xlsx
+++ b/src/OngGio.Infrastructure/Templates/BaoGiaExportTemplate.xlsx
@@ -185,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -247,6 +247,9 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -759,7 +762,7 @@
       <c r="I5" s="11" t="n"/>
       <c r="J5" s="11" t="n"/>
       <c r="K5" s="11" t="n"/>
-      <c r="L5" s="13" t="n"/>
+      <c r="L5" s="22" t="n"/>
       <c r="M5" s="14" t="n"/>
       <c r="N5" s="14" t="n"/>
       <c r="O5" s="15" t="n"/>

</xml_diff>